<commit_message>
auto: add club queens-park-rangers from TM URL (2026-06-08)
</commit_message>
<xml_diff>
--- a/data/sots_more_matches_confirmed.xlsx
+++ b/data/sots_more_matches_confirmed.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -471,15 +471,15 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Anass Salah-Eddine</t>
+          <t>Joe Walsh</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>485584</v>
+        <v>690548</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PSV</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -491,31 +491,31 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>37077855</v>
+        <v>29217723</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/37077855/anass-salah-eddine</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/29217723/joe-walsh</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2002-01-18</t>
+          <t>2002-04-01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Dailon Livramento</t>
+          <t>Paul Nardi</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>676411</v>
+        <v>189744</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Casa Pia</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -527,31 +527,31 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>37084655</v>
+        <v>85068996</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/37084655/dailon-livramento</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/85068996/paul-nardi</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2001-05-04</t>
+          <t>1994-05-18</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Saud Abdulhamid</t>
+          <t>Murphy Cooper</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>631927</v>
+        <v>921746</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Lens</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -563,31 +563,31 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>2000042460</v>
+        <v>29218345</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000042460/saud-abdulhamid</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/29218345/murphy-cooper</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1999-07-18</t>
+          <t>2001-12-27</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Stefan Posch</t>
+          <t>Ben Hamer</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>223974</v>
+        <v>67283</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Mainz</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -599,31 +599,31 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>16147386</v>
+        <v>5119981</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/16147386/stefan-posch</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/5119981/ben-hamer</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1997-05-14</t>
+          <t>1987-11-20</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Timothy Weah</t>
+          <t>Ronnie Edwards</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>370846</v>
+        <v>732165</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Marseille</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -635,31 +635,31 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>48042432</v>
+        <v>29243820</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/48042432/timothy-weah</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/29243820/ronnie-edwards</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2000-02-22</t>
+          <t>2003-03-28</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Noa Lang</t>
+          <t>Amadou Mbengue</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>339332</v>
+        <v>806310</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Galatasaray</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -671,31 +671,31 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>37055842</v>
+        <v>2000024506</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/37055842/noa-lang</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000024506/amadou-mbengue</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1999-06-17</t>
+          <t>2002-01-05</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Eldor Shomurodov</t>
+          <t>Liam Morrison</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>358166</v>
+        <v>567114</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Basaksehir</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -707,31 +707,31 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>59061760</v>
+        <v>61094579</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/59061760/eldor-shomurodov</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/61094579/liam-morrison</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1995-06-29</t>
+          <t>2003-04-07</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Nicola Bagnolini</t>
+          <t>Jake Clarke-Salter</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>818892</v>
+        <v>316551</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AS Gubbio</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -743,31 +743,31 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2000020964</v>
+        <v>28097983</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000020964/nicola-bagnolini</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/28097983/jake-clarke-salter</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2004-03-14</t>
+          <t>1997-09-22</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Titas Krapikas</t>
+          <t>Steve Cook</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>353609</v>
+        <v>90836</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AS Gubbio</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -779,31 +779,31 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>29157184</v>
+        <v>28014634</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/29157184/titas-krapikas</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/28014634/steve-cook</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1999-01-03</t>
+          <t>1991-04-19</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Leonardo Baroncelli</t>
+          <t>Esquerdinha</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>932733</v>
+        <v>1004737</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AS Gubbio</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -815,31 +815,31 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2000104785</v>
+        <v>2000218798</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000104785/leonardo-baroncelli</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000218798/esquerdinha</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2005-08-13</t>
+          <t>2006-02-28</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Alessandro Di Bitonto</t>
+          <t>Rhys Norrington-Davies</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>932763</v>
+        <v>543164</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AS Gubbio</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -851,31 +851,31 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>2000103801</v>
+        <v>29193986</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000103801/alessandro-di-bitonto</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/29193986/rhys-norrington-davies</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2005-10-08</t>
+          <t>1999-04-22</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Andrea Signorini</t>
+          <t>Ziyad Larkeche</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>56682</v>
+        <v>618402</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AS Gubbio</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -887,31 +887,31 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>43000523</v>
+        <v>49060914</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/43000523/andrea-signorini</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/49060914/ziyad-larkeche</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1990-01-31</t>
+          <t>2002-09-19</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Alberto Tentardini</t>
+          <t>Jimmy Dunne</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>281633</v>
+        <v>396174</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AS Gubbio</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -923,31 +923,31 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>43140548</v>
+        <v>28100270</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/43140548/alberto-tentardini</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/28100270/jimmy-dunne</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1996-10-21</t>
+          <t>1997-10-19</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Nicola Murru</t>
+          <t>Sam Field</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>171399</v>
+        <v>387331</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AS Gubbio</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -959,31 +959,31 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>43082118</v>
+        <v>28101021</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/43082118/nicola-murru</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/28101021/sam-field</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1994-12-16</t>
+          <t>1998-05-08</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Matteo Bruscagin</t>
+          <t>Jonathan Varane</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>56618</v>
+        <v>812902</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AS Gubbio</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -995,31 +995,31 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>43006835</v>
+        <v>49054406</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/43006835/matteo-bruscagin</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/49054406/jonathan-varane</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1989-08-03</t>
+          <t>2001-09-09</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Lorenzo Podda</t>
+          <t>Isaac Hayden</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>816897</v>
+        <v>206225</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AS Gubbio</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1031,31 +1031,31 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>43500641</v>
+        <v>28067790</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/43500641/lorenzo-podda</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/28067790/isaac-hayden</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2003-04-09</t>
+          <t>1995-03-22</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Francesco Zallu</t>
+          <t>Nicolas Madsen</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>711352</v>
+        <v>464599</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>AS Gubbio</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1067,31 +1067,31 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>43617805</v>
+        <v>27129144</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/43617805/francesco-zallu</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/27129144/nicolas-madsen</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2003-04-29</t>
+          <t>2000-03-17</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Nicolò Fazzi</t>
+          <t>Kieran Morgan</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>197744</v>
+        <v>1047344</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>AS Gubbio</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1103,31 +1103,31 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>43093494</v>
+        <v>2000222070</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/43093494/nicolo-fazzi</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000222070/kieran-morgan</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>1995-03-02</t>
+          <t>2006-03-17</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Federico Carraro</t>
+          <t>Harvey Vale</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>62718</v>
+        <v>581675</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>AS Gubbio</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1139,31 +1139,31 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>43009072</v>
+        <v>2000016607</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/43009072/federico-carraro</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000016607/harvey-vale</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1992-06-23</t>
+          <t>2003-09-11</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Halid Djankpata</t>
+          <t>Ilias Chair</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>924901</v>
+        <v>380473</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AS Gubbio</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1175,31 +1175,31 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2000134429</v>
+        <v>18089606</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000134429/halid-djankpata</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/18089606/ilias-chair</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2005-04-13</t>
+          <t>1997-10-30</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Ivan Varone</t>
+          <t>Koki Saito</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>123258</v>
+        <v>501743</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>AS Gubbio</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1211,31 +1211,31 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>43074244</v>
+        <v>45109986</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/43074244/ivan-varone</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/45109986/koki-saito</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>1992-10-11</t>
+          <t>2001-08-10</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Saber Hraiech</t>
+          <t>Daniel Bennie</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>256118</v>
+        <v>1104713</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>AS Gubbio</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -1247,31 +1247,31 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>43116070</v>
+        <v>2000089797</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/43116070/saber-hraiech</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000089797/daniel-bennie</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1995-07-30</t>
+          <t>2006-04-13</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Giacomo Rosaia</t>
+          <t>Kwame Poku</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>62750</v>
+        <v>701062</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>AS Gubbio</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1283,31 +1283,31 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>43084559</v>
+        <v>29228252</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/43084559/giacomo-rosaia</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/29228252/kwame-poku</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>1993-03-26</t>
+          <t>2001-08-11</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Gabriele Costa</t>
+          <t>Paul Smyth</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>819083</v>
+        <v>408872</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>AS Gubbio</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -1319,31 +1319,31 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2000021640</v>
+        <v>52079995</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000021640/gabriele-costa</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/52079995/paul-smyth</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2004-12-10</t>
+          <t>1997-09-10</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Valerio Conti</t>
+          <t>Richard Kone</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1297382</v>
+        <v>1218761</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>AS Gubbio</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1355,31 +1355,31 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>2000266768</v>
+        <v>2000108166</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000266768/valerio-conti</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000108166/richard-kone</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2006-04-16</t>
+          <t>2003-07-15</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Alessio Di Massimo</t>
+          <t>Rumarn Burrell</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>402114</v>
+        <v>624946</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>AS Gubbio</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1391,31 +1391,31 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>43202175</v>
+        <v>29186220</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/43202175/alessio-di-massimo</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/29186220/rumarn-burrell</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1996-05-07</t>
+          <t>2000-12-16</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Amoako Minta</t>
+          <t>Rayan Kolli</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1249656</v>
+        <v>867699</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>AS Gubbio</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1427,31 +1427,31 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2000350267</v>
+        <v>2000138737</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000350267/amoako-minta</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000138737/rayan-kolli</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>2005-10-26</t>
+          <t>2005-02-10</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Federico Mastropietro</t>
+          <t>Alfie Lloyd</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>386577</v>
+        <v>838926</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>AS Gubbio</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1463,88 +1463,16 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>43252862</v>
+        <v>225123</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/43252862/federico-mastropietro</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/225123/alfie-lloyd</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1999-01-23</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Tommaso Ghirardello</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>930944</v>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>AS Gubbio</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>slug_esatto</t>
-        </is>
-      </c>
-      <c r="F30" t="n">
-        <v>2000101154</v>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000101154/tommaso-ghirardello</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>2005-10-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Andrea La Mantia</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>134983</v>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>AS Gubbio</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
-        <v>1</v>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>slug_esatto</t>
-        </is>
-      </c>
-      <c r="F31" t="n">
-        <v>43061716</v>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/43061716/andrea-la-mantia</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>1991-05-06</t>
+          <t>2003-04-30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: add club queens-park-rangers from TM URL (2026-07-13)
</commit_message>
<xml_diff>
--- a/data/sots_more_matches_confirmed.xlsx
+++ b/data/sots_more_matches_confirmed.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -471,15 +471,15 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Antoni Mikułko</t>
+          <t>Matvey Safonov</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>826506</v>
+        <v>318470</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Wieczysta Krakow</t>
+          <t>PSG</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -491,31 +491,31 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>2000035772</v>
+        <v>58123738</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000035772/antoni-mikulko</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/58123738/matvey-safonov</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2005-02-11</t>
+          <t>1999-02-25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Daniel Mikolajewski</t>
+          <t>Lucas Chevalier</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>448567</v>
+        <v>463600</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Wieczysta Krakow</t>
+          <t>PSG</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -527,31 +527,31 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>96109884</v>
+        <v>49048357</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/96109884/daniel-mikolajewski</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/49048357/lucas-chevalier</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1999-08-25</t>
+          <t>2001-11-06</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Dawid Szymonowicz</t>
+          <t>Renato Marin</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>242846</v>
+        <v>1041614</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Wieczysta</t>
+          <t>PSG</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -563,31 +563,31 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>96063637</v>
+        <v>2000198858</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/96063637/dawid-szymonowicz</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000198858/renato-marin</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1995-07-07</t>
+          <t>2006-07-10</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Michal Koj</t>
+          <t>Senny Mayulu</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>185679</v>
+        <v>903693</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Wieczysta Krakow</t>
+          <t>PSG</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -599,31 +599,31 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>36044695</v>
+        <v>2000179713</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/36044695/michal-koj</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000179713/senny-mayulu</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1993-07-28</t>
+          <t>2006-05-17</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Michał Pazdan</t>
+          <t>Khvicha Kvaratskhelia</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>54512</v>
+        <v>502670</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Wieczysta Krakow</t>
+          <t>PSG</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -635,31 +635,31 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>54006273</v>
+        <v>59130638</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/54006273/michal-pazdan</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/59130638/khvicha-kvaratskhelia</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1987-09-21</t>
+          <t>2001-02-12</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Kamil Pestka</t>
+          <t>Quentin Ndjantou</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>384482</v>
+        <v>1053208</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Wieczysta</t>
+          <t>PSG</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -671,31 +671,31 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>96120625</v>
+        <v>2000288850</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/96120625/kamil-pestka</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000288850/quentin-ndjantou</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1998-08-22</t>
+          <t>2007-07-23</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Rafal Pietrzak</t>
+          <t>Lorenzo Lucca</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>74722</v>
+        <v>572265</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Wieczysta Krakow</t>
+          <t>Nott'm Forest</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -707,31 +707,31 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>54008755</v>
+        <v>43409366</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/54008755/rafal-pietrzak</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/43409366/lorenzo-lucca</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1992-01-30</t>
+          <t>2000-09-10</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Karol Fila</t>
+          <t>Caleb Okoli</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>385817</v>
+        <v>461833</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Wieczysta</t>
+          <t>Leicester</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -743,31 +743,31 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>96093091</v>
+        <v>43372285</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/96093091/karol-fila</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/43372285/caleb-okoli</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1998-06-13</t>
+          <t>2001-07-13</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Kamil Dankowski</t>
+          <t>Luca Reggiani</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>255085</v>
+        <v>1074990</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Wieczysta</t>
+          <t>Dortmund</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -779,31 +779,31 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>96053730</v>
+        <v>2000333549</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/96053730/kamil-dankowski</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000333549/luca-reggiani</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1996-07-22</t>
+          <t>2008-01-09</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Nikola Knezevic</t>
+          <t>Samuele Inácio</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>706511</v>
+        <v>1058359</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>OFK Beograd</t>
+          <t>Dortmund</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -815,31 +815,31 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2000076073</v>
+        <v>2000338374</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000076073/nikola-knezevic</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000338374/samuele-inacio</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2003-03-10</t>
+          <t>2008-04-02</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Mikkel Maigaard</t>
+          <t>Fabio Chiarodia</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>265545</v>
+        <v>724104</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Cracovia</t>
+          <t>Mönchengladbach</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -851,31 +851,31 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>27088084</v>
+        <v>2000116422</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/27088084/mikkel-maigaard</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000116422/fabio-chiarodia</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1995-09-20</t>
+          <t>2005-06-05</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Michal Trabka</t>
+          <t>Matías Moreno</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>288542</v>
+        <v>1144700</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Wieczysta Krakow</t>
+          <t>Fiorentina</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -887,31 +887,31 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>96075516</v>
+        <v>2000158335</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/96075516/michal-trabka</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000158335/matias-moreno</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1997-04-22</t>
+          <t>2003-09-24</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Jacek Góralski</t>
+          <t>Alessandro Perrotti</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>199297</v>
+        <v>1223890</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Wieczysta Krakow</t>
+          <t>Fiorentina U20</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -923,31 +923,31 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>96029863</v>
+        <v>2000442543</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/96029863/jacek-goralski</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000442543/alessandro-perrotti</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1992-09-21</t>
+          <t>2008-01-30</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Tomasz Swedrowski</t>
+          <t>Antonio Pirrò</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>266170</v>
+        <v>1078812</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Wieczysta Krakow</t>
+          <t>Fiorentina U20</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -959,31 +959,31 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>96032345</v>
+        <v>2000442528</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/96032345/tomasz-swedrowski</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000442528/antonio-pirro</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1993-11-25</t>
+          <t>2008-01-28</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Petar Pusic</t>
+          <t>Matteo Salamon</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>390169</v>
+        <v>879371</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Wieczysta</t>
+          <t>QPR U21</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -995,31 +995,31 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>98038309</v>
+        <v>2000081255</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/98038309/petar-pusic</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000081255/matteo-salamon</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1999-01-25</t>
+          <t>2004-02-18</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Lucas Piazón</t>
+          <t>Tylon Smith</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>176485</v>
+        <v>1245612</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Wieczysta</t>
+          <t>QPR U21</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1031,31 +1031,31 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>19128545</v>
+        <v>2000343484</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/19128545/lucas-piazon</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000343484/tylon-smith</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1994-01-20</t>
+          <t>2005-05-09</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Maciej Gajos</t>
+          <t>Noah McCann</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>236891</v>
+        <v>1089414</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Wieczysta</t>
+          <t>Central Coast</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1067,31 +1067,31 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>96002753</v>
+        <v>2000222682</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/96002753/maciej-gajos</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000222682/noah-mccann</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>1991-03-19</t>
+          <t>2005-09-01</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Tobiasz Mras</t>
+          <t>Jake Leahy</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1143675</v>
+        <v>1089411</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>LKS Goczalkowice-Zdroj</t>
+          <t>Without Club</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1103,31 +1103,31 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2000312736</v>
+        <v>2000222678</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000312736/tobiasz-mras</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000222678/jake-leahy</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2007-06-10</t>
+          <t>2006-01-17</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Jacky Donkor</t>
+          <t>Jaiden Putman</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>553217</v>
+        <v>1225604</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Wieczysta</t>
+          <t>QPR U21</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1139,31 +1139,31 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>18102160</v>
+        <v>2000308768</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/18102160/jacky-donkor</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000308768/jaiden-putman</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1998-11-12</t>
+          <t>2006-09-18</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Miki Villar</t>
+          <t>Elijah Dixon-Bonner</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>382970</v>
+        <v>433180</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Wieczysta</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1175,31 +1175,31 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>67228445</v>
+        <v>28115785</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/67228445/miki-villar</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/28115785/elijah-dixon-bonner</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>1996-09-19</t>
+          <t>2001-01-01</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Lisandro Semedo</t>
+          <t>Alfie Tuck</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>225431</v>
+        <v>1005850</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Wieczysta Krakow</t>
+          <t>Maidstone</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1211,31 +1211,31 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>55070288</v>
+        <v>2000222683</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/55070288/lisandro-semedo</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000222683/alfie-tuck</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>1996-03-12</t>
+          <t>2006-05-09</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Paulinho</t>
+          <t>Teddy Tarbotton</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>842718</v>
+        <v>1352650</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>SC Otelul Galati</t>
+          <t>QPR U21</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -1247,31 +1247,31 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>83137420</v>
+        <v>2000408756</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/83137420/paulinho</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000408756/teddy-tarbotton</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1999-09-21</t>
+          <t>2007-09-29</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Stefan Feiertag</t>
+          <t>Isak Alemayehu</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>404949</v>
+        <v>935469</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Wieczysta</t>
+          <t>QPR U21</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1283,31 +1283,31 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>16191210</v>
+        <v>2000169743</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/16191210/stefan-feiertag</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000169743/isak-alemayehu</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2001-12-18</t>
+          <t>2006-10-11</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Carlitos</t>
+          <t>Jaylan Pearman</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>228885</v>
+        <v>1104726</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Wieczysta</t>
+          <t>QPR U21</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -1319,31 +1319,31 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>67127224</v>
+        <v>2000248324</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/67127224/carlitos</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000248324/jaylan-pearman</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>1990-06-12</t>
+          <t>2006-04-18</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Paweł Kieszek</t>
+          <t>Emmerson Sutton</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>17592</v>
+        <v>1225600</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Pogon Grodzisk</t>
+          <t>QPR U21</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1355,31 +1355,31 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>717397</v>
+        <v>2000308764</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/717397/pawel-kieszek</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000308764/emmerson-sutton</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1984-04-16</t>
+          <t>2006-12-28</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Mikołaj Glacel</t>
+          <t>Kalen Brunson</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>929420</v>
+        <v>1373897</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>KTS Weszlo Warszawa</t>
+          <t>QPR U18</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1391,31 +1391,31 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2000405933</v>
+        <v>2000511769</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000405933/mikolaj-glacel</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000511769/kalen-brunson</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2004-12-27</t>
+          <t>2009-04-17</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Karol Noiszewski</t>
+          <t>Leon Scarlett</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>605107</v>
+        <v>1376840</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Pogon Grodzisk Mazowiecki</t>
+          <t>QPR U18</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1427,31 +1427,31 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>96143057</v>
+        <v>2000511773</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/96143057/karol-noiszewski</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000511773/leon-scarlett</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1999-11-13</t>
+          <t>2009-08-16</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Grzegorz Gulczyński</t>
+          <t>Ashley Trujillo</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>296832</v>
+        <v>1348063</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Pogon Grodzisk Mazowiecki</t>
+          <t>QPR U18</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1463,31 +1463,31 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>96064491</v>
+        <v>2000453540</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/96064491/grzegorz-gulczynski</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000453540/ashley-trujillo</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1996-01-26</t>
+          <t>2008-12-10</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Kacper Łoś</t>
+          <t>Zan Celar</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>528409</v>
+        <v>340427</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Pogon Grodzisk Mazowiecki</t>
+          <t>QPR</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1499,31 +1499,31 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>96162744</v>
+        <v>62189940</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/96162744/kacper-los</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/62189940/zan-celar</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>2000-03-29</t>
+          <t>1999-03-14</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Matheus Dias</t>
+          <t>Cian Dillon</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>602185</v>
+        <v>1068357</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Pogon Grodzisk Mazowiecki</t>
+          <t>QPR U21</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1535,376 +1535,16 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>62232616</v>
+        <v>2000215020</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/62232616/matheus-dias</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/2000215020/cian-dillon</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1997-07-16</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Kamil Kargulewicz</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>562606</v>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Pogon Grodzisk</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>1</v>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>slug_esatto</t>
-        </is>
-      </c>
-      <c r="F32" t="n">
-        <v>96145026</v>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/96145026/kamil-kargulewicz</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>2000-09-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Jakub Konstantyn</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>694477</v>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Pogon Grodzisk</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
-        <v>1</v>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>slug_esatto</t>
-        </is>
-      </c>
-      <c r="F33" t="n">
-        <v>2000059430</v>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000059430/jakub-konstantyn</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>2002-06-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Jakub Niewiadomski</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>554970</v>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Pogon Grodzisk Mazowiecki</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>1</v>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>slug_esatto</t>
-        </is>
-      </c>
-      <c r="F34" t="n">
-        <v>96133801</v>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/96133801/jakub-niewiadomski</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>2002-04-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Olivier Wypart</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>605745</v>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Pogon Grodzisk</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>1</v>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>slug_esatto</t>
-        </is>
-      </c>
-      <c r="F35" t="n">
-        <v>96142655</v>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/96142655/olivier-wypart</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>2001-01-16</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Jakub Jędrasik</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>848943</v>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Pogon Grodzisk</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
-        <v>1</v>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>slug_esatto</t>
-        </is>
-      </c>
-      <c r="F36" t="n">
-        <v>2000177487</v>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000177487/jakub-jedrasik</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>2005-04-07</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Igor Korczakowski</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>385765</v>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Pogon Grodzisk Mazowiecki</t>
-        </is>
-      </c>
-      <c r="D37" t="n">
-        <v>1</v>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>slug_esatto</t>
-        </is>
-      </c>
-      <c r="F37" t="n">
-        <v>96127039</v>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/96127039/igor-korczakowski</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>1998-09-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Jakub Lis</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>1165401</v>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Pogon Grodzisk Mazowiecki</t>
-        </is>
-      </c>
-      <c r="D38" t="n">
-        <v>1</v>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>slug_esatto</t>
-        </is>
-      </c>
-      <c r="F38" t="n">
-        <v>2000396614</v>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000396614/jakub-lis</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>2004-10-14</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Hubert Adamczyk</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>287235</v>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Zaglebie Lubin</t>
-        </is>
-      </c>
-      <c r="D39" t="n">
-        <v>1</v>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>slug_esatto</t>
-        </is>
-      </c>
-      <c r="F39" t="n">
-        <v>28100044</v>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/28100044/hubert-adamczyk</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>1998-02-23</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Riccardo Calafiori</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>502821</v>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Arsenal</t>
-        </is>
-      </c>
-      <c r="D40" t="n">
-        <v>1</v>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>slug_esatto</t>
-        </is>
-      </c>
-      <c r="F40" t="n">
-        <v>43424738</v>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/43424738/riccardo-calafiori</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>2002-05-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Matteo Ruggeri</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>616631</v>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Atlético</t>
-        </is>
-      </c>
-      <c r="D41" t="n">
-        <v>1</v>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>slug_esatto</t>
-        </is>
-      </c>
-      <c r="F41" t="n">
-        <v>43425834</v>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/43425834/matteo-ruggeri</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>2002-07-11</t>
+          <t>2006-04-04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: add club deportivo-la-coruna from TM URL (2026-07-14)
</commit_message>
<xml_diff>
--- a/data/sots_more_matches_confirmed.xlsx
+++ b/data/sots_more_matches_confirmed.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -471,15 +471,15 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Andriy Lunin</t>
+          <t>Daniel Bachmann</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>404839</v>
+        <v>120186</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Real Madrid</t>
+          <t>Watford</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -491,31 +491,31 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>71099053</v>
+        <v>16045707</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/71099053/andriy-lunin</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/16045707/daniel-bachmann</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1999-02-11</t>
+          <t>1994-07-09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Dean Huijsen</t>
+          <t>José Gragera</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>890290</v>
+        <v>557147</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Real Madrid</t>
+          <t>Espanyol</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -527,31 +527,31 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>2000109240</v>
+        <v>67263880</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000109240/dean-huijsen</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/67263880/jose-gragera</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2005-04-14</t>
+          <t>2000-05-14</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Éder Militão</t>
+          <t>Samuele Mulattieri</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>401530</v>
+        <v>457422</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Real Madrid</t>
+          <t>Sassuolo</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -563,340 +563,16 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>19273276</v>
+        <v>43390644</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/19273276/eder-militao</t>
+          <t>https://sortitoutsi.net/football-manager-2026/person/43390644/samuele-mulattieri</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1998-01-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Raúl Asencio</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>935245</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Real Madrid</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>slug_esatto</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>2000126407</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000126407/raul-asencio</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2003-02-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Álvaro Carreras</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>811778</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Real Madrid</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>slug_esatto</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>2000032706</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000032706/alvaro-carreras</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>2003-03-23</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Fran García</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>341264</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Real Betis</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>slug_esatto</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>67245235</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/67245235/fran-garcia</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>1999-08-14</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Ferland Mendy</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>291417</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Real Madrid</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>slug_esatto</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>85133751</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/85133751/ferland-mendy</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>1995-06-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Trent Alexander-Arnold</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>314353</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Real Madrid</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>slug_esatto</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>28104124</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/28104124/trent-alexander-arnold</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>1998-10-07</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Eduardo Camavinga</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>640428</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Real Madrid</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>slug_esatto</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>49056243</v>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/49056243/eduardo-camavinga</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>2002-11-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Dani Ceballos</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>319745</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Without Club</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>slug_esatto</t>
-        </is>
-      </c>
-      <c r="F11" t="n">
-        <v>67202350</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/67202350/dani-ceballos</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>1996-08-07</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Rodrygo</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>412363</v>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Real Madrid</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>slug_esatto</t>
-        </is>
-      </c>
-      <c r="F12" t="n">
-        <v>19306929</v>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/19306929/rodrygo</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>2001-01-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Franco Mastantuono</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>1057316</v>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Real Madrid</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>slug_esatto</t>
-        </is>
-      </c>
-      <c r="F13" t="n">
-        <v>2000183231</v>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>https://sortitoutsi.net/football-manager-2026/person/2000183231/franco-mastantuono</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>2007-08-14</t>
+          <t>2000-10-07</t>
         </is>
       </c>
     </row>

</xml_diff>